<commit_message>
Migrate ep2 conte to telop notation v2; refine + rule in validator
- 21 cuts rewritten (★ prefixes dropped, 《》emphasis markers,
  in-graph labels tagged, C44 three points spelled out from narration)
- 22 mechanical S1/字幕全文 -> S1/全文 replacements
- validator: allow "+" followed by digits (e.g. +20%), still flag
  concatenation; both workbooks now pass with zero violations
- テロップ記法v2 sheet added to ep2 workbook; change log saved

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/第2回_コンテ表_v1.xlsx
+++ b/第2回_コンテ表_v1.xlsx
@@ -12,6 +12,7 @@
     <sheet name="BGM_SUNO" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="SE一覧" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="テロップ規定" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="テロップ記法v2" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MG制作計画'!$A$1:$M$38</definedName>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
@@ -81,6 +82,10 @@
       <b val="1"/>
       <color rgb="001A1A1A"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font/>
   </fonts>
   <fills count="13">
     <fill>
@@ -172,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -246,6 +251,8 @@
     <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -1041,14 +1048,18 @@
           <t>カット尻で全ポスト微ズーム寄り→C02へハードカット</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>S6/ポスト文言そのもの(は? 等)</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1件ごとにスケール105→100%のドン付き出現 [maxchar:12]</t>
+      <c r="P2" s="22" t="inlineStr">
+        <is>
+          <t>S6/は?
+S6/ありえない
+S6/拡散希望</t>
+        </is>
+      </c>
+      <c r="Q2" s="22" t="inlineStr">
+        <is>
+          <t>1件ごとにスケール105→100%のドン付き出現 [maxchar:12] [role:in-thumb] #架空ポスト画像内の文言
+〃
+〃</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -1166,7 +1177,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -1288,7 +1299,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1530,9 +1541,9 @@
           <t>紙フラッシュ→UIモックへ</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>S2/★不安の、その先へ。</t>
+      <c r="P6" s="22" t="inlineStr">
+        <is>
+          <t>S2/不安の、その先へ。</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1655,7 +1666,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1778,7 +1789,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1900,7 +1911,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -2020,14 +2031,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>S2/★あなたの怒りには、値段がついている。</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>★文:中央。「値段」のみ金茶1.2倍</t>
+      <c r="P10" s="22" t="inlineStr">
+        <is>
+          <t>S2/あなたの怒りには、《値段》がついている。</t>
+        </is>
+      </c>
+      <c r="Q10" s="22" t="inlineStr">
+        <is>
+          <t>★文:中央 [emph:値段|金茶,1.2倍]</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -2142,14 +2153,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>S4/怒りは、燃料になる(タイトル内)</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="P11" s="22" t="inlineStr">
+        <is>
+          <t>S4/怒りは、燃料になる</t>
+        </is>
+      </c>
+      <c r="Q11" s="22" t="inlineStr">
+        <is>
+          <t>[role:title]</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -2266,14 +2277,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>S2/★怒りは、感情ではなく燃料です。</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>★文:中央。「燃料」のみ金茶+1.2倍</t>
+      <c r="P12" s="22" t="inlineStr">
+        <is>
+          <t>S2/怒りは、感情ではなく《燃料》です。</t>
+        </is>
+      </c>
+      <c r="Q12" s="22" t="inlineStr">
+        <is>
+          <t>★文:中央 [emph:燃料|金茶,1.2倍]</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -2388,14 +2399,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>S5/+20%(数字)/1語ごとに(和文)</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>数字カウントアップ、棒はインク質感で伸長</t>
+      <c r="P13" s="22" t="inlineStr">
+        <is>
+          <t>S5/+20%
+S5/1語ごとに</t>
+        </is>
+      </c>
+      <c r="Q13" s="22" t="inlineStr">
+        <is>
+          <t>数字カウントアップ、棒はインク質感で伸長 [role:in-graph]
+〃</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -2511,9 +2524,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>S2/★回っているのは、広告です。</t>
+      <c r="P14" s="22" t="inlineStr">
+        <is>
+          <t>S2/回っているのは、広告です。</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -2633,14 +2646,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>S1/字幕全文(Before/Afterに同期)</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="P15" s="22" t="inlineStr">
+        <is>
+          <t>S1/全文</t>
+        </is>
+      </c>
+      <c r="Q15" s="22" t="inlineStr">
+        <is>
+          <t>[sync:Before/Afterの切替]</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2755,14 +2768,16 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>S5/×5(数字)/いいねの5倍(和文)</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>等式が順に出現、×5のみ朱</t>
+      <c r="P16" s="22" t="inlineStr">
+        <is>
+          <t>S5/×5
+S5/いいねの5倍</t>
+        </is>
+      </c>
+      <c r="Q16" s="22" t="inlineStr">
+        <is>
+          <t>等式が順に出現 [role:in-graph] [emph:×5|朱]
+〃</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -3001,7 +3016,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -3121,9 +3136,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>S2/★怒りっぽさは、性格ではなく学習です。</t>
+      <c r="P19" s="22" t="inlineStr">
+        <is>
+          <t>S2/怒りっぽさは、性格ではなく《学習》です。</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -3245,7 +3260,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -3366,9 +3381,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>S2/★わざと嫌われている人が、います。</t>
+      <c r="P21" s="22" t="inlineStr">
+        <is>
+          <t>S2/わざと嫌われている人が、います。</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -3490,7 +3505,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -3856,7 +3871,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -3977,9 +3992,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>S2/★売っていたのは「興奮」です。</t>
+      <c r="P26" s="22" t="inlineStr">
+        <is>
+          <t>S2/売っていたのは「興奮」です。</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -4101,7 +4116,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -4345,7 +4360,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -4465,9 +4480,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>S2/★他人の怒りが、商品になった。</t>
+      <c r="P30" s="22" t="inlineStr">
+        <is>
+          <t>S2/他人の怒りが、商品になった。</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -4590,7 +4605,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -4710,9 +4725,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>S2/★怒る相手は、機械が選んでいる。</t>
+      <c r="P32" s="22" t="inlineStr">
+        <is>
+          <t>S2/怒る相手は、機械が選んでいる。</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -4834,7 +4849,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -4957,7 +4972,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -5079,7 +5094,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -5199,9 +5214,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>S2/★怒りは、いちばん安い燃料。</t>
+      <c r="P36" s="22" t="inlineStr">
+        <is>
+          <t>S2/怒りは、いちばん安い燃料。</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -5323,7 +5338,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -5443,9 +5458,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>S2/★わざと嫌われている人が、います。</t>
+      <c r="P38" s="22" t="inlineStr">
+        <is>
+          <t>S2/わざと嫌われている人が、います。</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -5567,7 +5582,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -5810,14 +5825,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>S5/¥(数字)/表示回数→収益(和文)</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>カウントアップ→¥変換で朱が一瞬差す</t>
+      <c r="P41" s="22" t="inlineStr">
+        <is>
+          <t>S5/表示回数→収益</t>
+        </is>
+      </c>
+      <c r="Q41" s="22" t="inlineStr">
+        <is>
+          <t>カウントアップ→¥変換で朱が一瞬差す [role:in-graph]</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -5934,7 +5949,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -6054,9 +6069,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>S2/★いちばん静かに得をしている人は、誰か。</t>
+      <c r="P43" s="22" t="inlineStr">
+        <is>
+          <t>S2/いちばん静かに得をしている人は、誰か。</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -6179,7 +6194,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -6301,14 +6316,18 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>S2/★3点(順次)</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>順に積む。各行の強調語のみ金茶</t>
+      <c r="P45" s="22" t="inlineStr">
+        <is>
+          <t>S2/ひとつ。怒りは、いちばん速く広がって、いちばん安くつく《燃料》です。
+S2/ふたつ。あなたが怒る相手は、《機械》が、あなた専用に選んでいます。
+S2/みっつ。あなたの怒りのリプライは、燃やした本人の《売上》になります。</t>
+        </is>
+      </c>
+      <c r="Q45" s="22" t="inlineStr">
+        <is>
+          <t>順に積む(第1回C48と同一機構) [pos:left] [seq:順次]
+〃
+〃</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -6425,7 +6444,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -6545,9 +6564,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>S2/★怒りの行き先は、自分で決める。</t>
+      <c r="P47" s="22" t="inlineStr">
+        <is>
+          <t>S2/怒りの行き先は、自分で決める。</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -6670,7 +6689,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -6795,9 +6814,9 @@
           <t>S4/『なんだろう』解体</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="Q49" s="22" t="inlineStr">
+        <is>
+          <t>[role:logo]</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -6914,7 +6933,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -7036,14 +7055,14 @@
           <t>—</t>
         </is>
       </c>
-      <c r="P51" t="inlineStr">
-        <is>
-          <t>S2/★次回:「おすすめ」はなぜ当たるのか(仮)</t>
-        </is>
-      </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>M6規定+粒子</t>
+      <c r="P51" s="22" t="inlineStr">
+        <is>
+          <t>S2/『おすすめ』は、なぜ、あなたの好みを知っているのか</t>
+        </is>
+      </c>
+      <c r="Q51" s="22" t="inlineStr">
+        <is>
+          <t>M6規定+粒子 [role:next-title] #次回テーマは仮。確定後に差し替え</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -10861,4 +10880,266 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>テロップ記法 v2(2026-07-13制定)</t>
+        </is>
+      </c>
+      <c r="B1" s="22" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr"/>
+      <c r="B2" s="22" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>■ テロップ列(スタイル/内容)のルール</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>1行 = 1テロップ。書式は「Sn/本文」(nは1〜6)。欧文は「Sn(欧文)/本文」</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>本文には画面に出す文字だけを書く。制作指示・位置・演出メモは書かない(モーション列へ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>特殊値「S1/全文」= ナレーション列の全文を字幕にする(旧「字幕全文」)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>強調語は本文中で《》で括る。例: S2/不安は、商品ではありません。《エサです。》 デフォルトの強調=金茶</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>複数テロップは改行して並べる。順次表示もスタイルを行ごとに繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>禁止: 「+」での連結(+数字は可) / (括弧)での指示 / 「〜のみ金茶」「併走」「画面主役」等の指示文の混入</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr"/>
+      <c r="B10" s="22" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>■ モーション列のルール</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>テロップ列の行と同順で1行ずつ対応させる。同じ内容の繰り返しは「〃」</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>構造化タグ: [pos:位置] [offset:x,y] [maxchar:n] [sync:同期先] [seq:順次] [role:役割] [emph:語|効果]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>[emph:語|効果] は金茶以外の強調(色同期・サイズ変更・字間など)を指定する</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>[role:] の値: title / logo / next-title / in-thumb / in-image / in-graph / in-demo(画面内合成を示す)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>「#」以降は自由メモ(機械処理の対象外)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr"/>
+      <c r="B17" s="22" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>■ スタイル別の管理先</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>標準字幕。Premiere SRT(conte2srt.py)で管理。Remotionオーバーレイの対象外</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>S2/S3/S5</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>RemotionのTelopOverlayで生成(透過mov)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>黒画面宣言はオーバーレイではなくフルフレームカット。JsonScenesのstatement型で作る</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>サムネ/ポスト画像内の文字。Canva/Photoshop側で制作(オーバーレイ対象外)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr"/>
+      <c r="B23" s="22" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>■ 検証</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr"/>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>python3 validate_telops.py &lt;コンテ表.xlsx&gt; で違反を検出。警告ゼロにしてから変換に進む</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>